<commit_message>
update data GNI pc
</commit_message>
<xml_diff>
--- a/xlsx/'folder' missing.xlsx
+++ b/xlsx/'folder' missing.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="146" uniqueCount="146">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="178" uniqueCount="178">
   <si>
     <t xml:space="preserve"/>
   </si>
@@ -26,15 +26,24 @@
     <t xml:space="preserve">Albania</t>
   </si>
   <si>
+    <t xml:space="preserve">United Arab Emirates</t>
+  </si>
+  <si>
     <t xml:space="preserve">Argentina</t>
   </si>
   <si>
     <t xml:space="preserve">Armenia</t>
   </si>
   <si>
+    <t xml:space="preserve">Australia</t>
+  </si>
+  <si>
     <t xml:space="preserve">Austria</t>
   </si>
   <si>
+    <t xml:space="preserve">Azerbaijan</t>
+  </si>
+  <si>
     <t xml:space="preserve">Burundi</t>
   </si>
   <si>
@@ -53,12 +62,18 @@
     <t xml:space="preserve">Bulgaria</t>
   </si>
   <si>
+    <t xml:space="preserve">Bahrain</t>
+  </si>
+  <si>
     <t xml:space="preserve">Bahamas</t>
   </si>
   <si>
     <t xml:space="preserve">Bosnia and Herzegovina</t>
   </si>
   <si>
+    <t xml:space="preserve">Belarus</t>
+  </si>
+  <si>
     <t xml:space="preserve">Belize</t>
   </si>
   <si>
@@ -71,6 +86,9 @@
     <t xml:space="preserve">Barbados</t>
   </si>
   <si>
+    <t xml:space="preserve">Brunei</t>
+  </si>
+  <si>
     <t xml:space="preserve">Bhutan</t>
   </si>
   <si>
@@ -80,6 +98,9 @@
     <t xml:space="preserve">Central African Republic</t>
   </si>
   <si>
+    <t xml:space="preserve">Canada</t>
+  </si>
+  <si>
     <t xml:space="preserve">Switzerland</t>
   </si>
   <si>
@@ -158,6 +179,9 @@
     <t xml:space="preserve">Finland</t>
   </si>
   <si>
+    <t xml:space="preserve">Fiji</t>
+  </si>
+  <si>
     <t xml:space="preserve">France</t>
   </si>
   <si>
@@ -194,6 +218,9 @@
     <t xml:space="preserve">Guyana</t>
   </si>
   <si>
+    <t xml:space="preserve">Hong Kong</t>
+  </si>
+  <si>
     <t xml:space="preserve">Honduras</t>
   </si>
   <si>
@@ -224,6 +251,9 @@
     <t xml:space="preserve">Iceland</t>
   </si>
   <si>
+    <t xml:space="preserve">Israel</t>
+  </si>
+  <si>
     <t xml:space="preserve">Italy</t>
   </si>
   <si>
@@ -236,18 +266,30 @@
     <t xml:space="preserve">Japan</t>
   </si>
   <si>
+    <t xml:space="preserve">Kazakhstan</t>
+  </si>
+  <si>
     <t xml:space="preserve">Kenya</t>
   </si>
   <si>
+    <t xml:space="preserve">Kyrgyzstan</t>
+  </si>
+  <si>
     <t xml:space="preserve">Cambodia</t>
   </si>
   <si>
     <t xml:space="preserve">South Korea</t>
   </si>
   <si>
+    <t xml:space="preserve">Kuwait</t>
+  </si>
+  <si>
     <t xml:space="preserve">Laos</t>
   </si>
   <si>
+    <t xml:space="preserve">Lebanon</t>
+  </si>
+  <si>
     <t xml:space="preserve">Liberia</t>
   </si>
   <si>
@@ -284,6 +326,9 @@
     <t xml:space="preserve">Mexico</t>
   </si>
   <si>
+    <t xml:space="preserve">North Macedonia</t>
+  </si>
+  <si>
     <t xml:space="preserve">Mali</t>
   </si>
   <si>
@@ -293,6 +338,9 @@
     <t xml:space="preserve">Myanmar</t>
   </si>
   <si>
+    <t xml:space="preserve">Montenegro</t>
+  </si>
+  <si>
     <t xml:space="preserve">Mongolia</t>
   </si>
   <si>
@@ -332,6 +380,12 @@
     <t xml:space="preserve">Nepal</t>
   </si>
   <si>
+    <t xml:space="preserve">New Zealand</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Oman</t>
+  </si>
+  <si>
     <t xml:space="preserve">Pakistan</t>
   </si>
   <si>
@@ -350,18 +404,30 @@
     <t xml:space="preserve">Poland</t>
   </si>
   <si>
+    <t xml:space="preserve">North Korea</t>
+  </si>
+  <si>
     <t xml:space="preserve">Portugal</t>
   </si>
   <si>
     <t xml:space="preserve">Paraguay</t>
   </si>
   <si>
+    <t xml:space="preserve">Qatar</t>
+  </si>
+  <si>
     <t xml:space="preserve">Romania</t>
   </si>
   <si>
+    <t xml:space="preserve">Russia</t>
+  </si>
+  <si>
     <t xml:space="preserve">Rwanda</t>
   </si>
   <si>
+    <t xml:space="preserve">Saudi Arabia</t>
+  </si>
+  <si>
     <t xml:space="preserve">Sudan</t>
   </si>
   <si>
@@ -371,15 +437,24 @@
     <t xml:space="preserve">Singapore</t>
   </si>
   <si>
+    <t xml:space="preserve">Solomon Islands</t>
+  </si>
+  <si>
     <t xml:space="preserve">Sierra Leone</t>
   </si>
   <si>
     <t xml:space="preserve">El Salvador</t>
   </si>
   <si>
+    <t xml:space="preserve">Somalia</t>
+  </si>
+  <si>
     <t xml:space="preserve">Serbia</t>
   </si>
   <si>
+    <t xml:space="preserve">South Sudan</t>
+  </si>
+  <si>
     <t xml:space="preserve">Suriname</t>
   </si>
   <si>
@@ -407,18 +482,27 @@
     <t xml:space="preserve">Thailand</t>
   </si>
   <si>
+    <t xml:space="preserve">Tajikistan</t>
+  </si>
+  <si>
     <t xml:space="preserve">Turkmenistan</t>
   </si>
   <si>
     <t xml:space="preserve">Timor</t>
   </si>
   <si>
+    <t xml:space="preserve">Trinidad and Tobago</t>
+  </si>
+  <si>
     <t xml:space="preserve">Tunisia</t>
   </si>
   <si>
     <t xml:space="preserve">Turkey</t>
   </si>
   <si>
+    <t xml:space="preserve">Taiwan</t>
+  </si>
+  <si>
     <t xml:space="preserve">Tanzania</t>
   </si>
   <si>
@@ -431,12 +515,24 @@
     <t xml:space="preserve">Uruguay</t>
   </si>
   <si>
+    <t xml:space="preserve">USA</t>
+  </si>
+  <si>
     <t xml:space="preserve">Uzbekistan</t>
   </si>
   <si>
+    <t xml:space="preserve">Venezuela</t>
+  </si>
+  <si>
     <t xml:space="preserve">Vietnam</t>
   </si>
   <si>
+    <t xml:space="preserve">Vanuatu</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Samoa</t>
+  </si>
+  <si>
     <t xml:space="preserve">Yemen</t>
   </si>
   <si>
@@ -449,7 +545,7 @@
     <t xml:space="preserve">Zimbabwe</t>
   </si>
   <si>
-    <t xml:space="preserve">diff_ede_cs_bau</t>
+    <t xml:space="preserve">net_gain_over_gdp_both_taxes</t>
   </si>
 </sst>
 </file>
@@ -1214,442 +1310,630 @@
       <c r="EO1" t="s">
         <v>144</v>
       </c>
+      <c r="EP1" t="s">
+        <v>145</v>
+      </c>
+      <c r="EQ1" t="s">
+        <v>146</v>
+      </c>
+      <c r="ER1" t="s">
+        <v>147</v>
+      </c>
+      <c r="ES1" t="s">
+        <v>148</v>
+      </c>
+      <c r="ET1" t="s">
+        <v>149</v>
+      </c>
+      <c r="EU1" t="s">
+        <v>150</v>
+      </c>
+      <c r="EV1" t="s">
+        <v>151</v>
+      </c>
+      <c r="EW1" t="s">
+        <v>152</v>
+      </c>
+      <c r="EX1" t="s">
+        <v>153</v>
+      </c>
+      <c r="EY1" t="s">
+        <v>154</v>
+      </c>
+      <c r="EZ1" t="s">
+        <v>155</v>
+      </c>
+      <c r="FA1" t="s">
+        <v>156</v>
+      </c>
+      <c r="FB1" t="s">
+        <v>157</v>
+      </c>
+      <c r="FC1" t="s">
+        <v>158</v>
+      </c>
+      <c r="FD1" t="s">
+        <v>159</v>
+      </c>
+      <c r="FE1" t="s">
+        <v>160</v>
+      </c>
+      <c r="FF1" t="s">
+        <v>161</v>
+      </c>
+      <c r="FG1" t="s">
+        <v>162</v>
+      </c>
+      <c r="FH1" t="s">
+        <v>163</v>
+      </c>
+      <c r="FI1" t="s">
+        <v>164</v>
+      </c>
+      <c r="FJ1" t="s">
+        <v>165</v>
+      </c>
+      <c r="FK1" t="s">
+        <v>166</v>
+      </c>
+      <c r="FL1" t="s">
+        <v>167</v>
+      </c>
+      <c r="FM1" t="s">
+        <v>168</v>
+      </c>
+      <c r="FN1" t="s">
+        <v>169</v>
+      </c>
+      <c r="FO1" t="s">
+        <v>170</v>
+      </c>
+      <c r="FP1" t="s">
+        <v>171</v>
+      </c>
+      <c r="FQ1" t="s">
+        <v>172</v>
+      </c>
+      <c r="FR1" t="s">
+        <v>173</v>
+      </c>
+      <c r="FS1" t="s">
+        <v>174</v>
+      </c>
+      <c r="FT1" t="s">
+        <v>175</v>
+      </c>
+      <c r="FU1" t="s">
+        <v>176</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>145</v>
+        <v>177</v>
       </c>
       <c r="B2" t="n">
-        <v>0.0960242610498829</v>
+        <v>0.410971735578937</v>
       </c>
       <c r="C2" t="n">
-        <v>0.0959752570803243</v>
+        <v>0.0597841880274297</v>
       </c>
       <c r="D2" t="n">
-        <v>0.00611961280230622</v>
+        <v>0.0152364997229248</v>
       </c>
       <c r="E2" t="n">
-        <v>0.0060634451538677</v>
+        <v>-0.0087596161924643</v>
       </c>
       <c r="F2" t="n">
-        <v>0.0065092089808696</v>
+        <v>0.00125382801828126</v>
       </c>
       <c r="G2" t="n">
-        <v>-0.00745990614656611</v>
+        <v>0.0180110018613807</v>
       </c>
       <c r="H2" t="n">
-        <v>0.172955752391303</v>
+        <v>-0.00996254235275846</v>
       </c>
       <c r="I2" t="n">
-        <v>-0.0216771845038177</v>
+        <v>-0.00979995269691796</v>
       </c>
       <c r="J2" t="n">
-        <v>0.0916140579861662</v>
+        <v>0.0174298289588247</v>
       </c>
       <c r="K2" t="n">
-        <v>0.115182025322397</v>
+        <v>0.691111495278733</v>
       </c>
       <c r="L2" t="n">
-        <v>0.0277748798714754</v>
+        <v>-0.00754893718787074</v>
       </c>
       <c r="M2" t="n">
-        <v>-0.000194441770287823</v>
+        <v>0.10370630023442</v>
       </c>
       <c r="N2" t="n">
-        <v>0.00695000026225823</v>
+        <v>0.172356569311058</v>
       </c>
       <c r="O2" t="n">
-        <v>-0.0340767121784475</v>
+        <v>0.0596599519032092</v>
       </c>
       <c r="P2" t="n">
-        <v>0.081439782269296</v>
+        <v>0.000991924056784935</v>
       </c>
       <c r="Q2" t="n">
-        <v>0.0151415341665564</v>
+        <v>-0.00804665496508791</v>
       </c>
       <c r="R2" t="n">
-        <v>0.0616821629292419</v>
+        <v>-0.00890288128693816</v>
       </c>
       <c r="S2" t="n">
-        <v>0.0176577463997194</v>
+        <v>0.0134179109489133</v>
       </c>
       <c r="T2" t="n">
-        <v>0.00195943736368354</v>
+        <v>0.0147160573770233</v>
       </c>
       <c r="U2" t="n">
-        <v>0.101664719841149</v>
+        <v>0.0144875217301594</v>
       </c>
       <c r="V2" t="n">
-        <v>0.468009267714899</v>
+        <v>0.0394247015544232</v>
       </c>
       <c r="W2" t="n">
-        <v>-0.0170292220616327</v>
+        <v>0.00833668573562733</v>
       </c>
       <c r="X2" t="n">
-        <v>0.00682492695399195</v>
+        <v>-0.00595225655433289</v>
       </c>
       <c r="Y2" t="n">
-        <v>-0.008576176594564</v>
+        <v>-0.00919761683212933</v>
       </c>
       <c r="Z2" t="n">
-        <v>0.0439445644559844</v>
+        <v>0.0460314326566047</v>
       </c>
       <c r="AA2" t="n">
-        <v>0.0791741444624203</v>
+        <v>0.00787605735485338</v>
       </c>
       <c r="AB2" t="n">
-        <v>0.123984288043975</v>
+        <v>0.265972069702707</v>
       </c>
       <c r="AC2" t="n">
-        <v>0.0672542159979814</v>
+        <v>-0.0101327721372749</v>
       </c>
       <c r="AD2" t="n">
-        <v>0.0458315339684319</v>
+        <v>-0.0126155460514852</v>
       </c>
       <c r="AE2" t="n">
-        <v>0.201685603243885</v>
+        <v>-0.00134251304472625</v>
       </c>
       <c r="AF2" t="n">
-        <v>0.0572300157181291</v>
+        <v>-0.000913763029050369</v>
       </c>
       <c r="AG2" t="n">
-        <v>0.0105193754873296</v>
+        <v>0.0529696088544215</v>
       </c>
       <c r="AH2" t="n">
-        <v>0.00947520006068769</v>
+        <v>0.0831723982964351</v>
       </c>
       <c r="AI2" t="n">
-        <v>0.00167817652248559</v>
+        <v>0.228105664173023</v>
       </c>
       <c r="AJ2" t="n">
-        <v>-0.0128869324864236</v>
+        <v>0.0543303472902626</v>
       </c>
       <c r="AK2" t="n">
-        <v>-0.00711768269476165</v>
+        <v>0.017266303394593</v>
       </c>
       <c r="AL2" t="n">
-        <v>0.0804098038607584</v>
+        <v>0.0953003868124647</v>
       </c>
       <c r="AM2" t="n">
-        <v>-0.00564136505508195</v>
+        <v>0.0286829687472111</v>
       </c>
       <c r="AN2" t="n">
-        <v>0.0338205547649848</v>
+        <v>0.0000267980378655588</v>
       </c>
       <c r="AO2" t="n">
-        <v>0.00894006982703099</v>
+        <v>-0.000316596826565653</v>
       </c>
       <c r="AP2" t="n">
-        <v>0.00908157241898122</v>
+        <v>-0.00865664660174971</v>
       </c>
       <c r="AQ2" t="n">
-        <v>0.00820203733097591</v>
+        <v>-0.00775332834173738</v>
       </c>
       <c r="AR2" t="n">
-        <v>0.485956022784829</v>
+        <v>-0.00964180879415704</v>
       </c>
       <c r="AS2" t="n">
-        <v>0.000892405538883256</v>
+        <v>0.0431230816015328</v>
       </c>
       <c r="AT2" t="n">
-        <v>-0.0199654777490027</v>
+        <v>-0.0108834249140328</v>
       </c>
       <c r="AU2" t="n">
-        <v>0.0617937692109494</v>
+        <v>0.00592604978356308</v>
       </c>
       <c r="AV2" t="n">
-        <v>-0.010214925428934</v>
+        <v>0.0251730264741292</v>
       </c>
       <c r="AW2" t="n">
-        <v>-0.00247037517420234</v>
+        <v>0.0167047195329141</v>
       </c>
       <c r="AX2" t="n">
-        <v>0.0313277257247468</v>
+        <v>0.0350914754796716</v>
       </c>
       <c r="AY2" t="n">
-        <v>-0.00579282957333804</v>
+        <v>0.250552860323458</v>
       </c>
       <c r="AZ2" t="n">
-        <v>0.00113291541613059</v>
+        <v>-0.00646300197503676</v>
       </c>
       <c r="BA2" t="n">
-        <v>0.0707291194797013</v>
+        <v>-0.00769696895552049</v>
       </c>
       <c r="BB2" t="n">
-        <v>0.0745887757889936</v>
+        <v>0.140042535903052</v>
       </c>
       <c r="BC2" t="n">
-        <v>0.165507537106996</v>
+        <v>-0.0079483549662656</v>
       </c>
       <c r="BD2" t="n">
-        <v>0.165735819020308</v>
+        <v>0.0205633837666241</v>
       </c>
       <c r="BE2" t="n">
-        <v>0.0272019456457899</v>
+        <v>-0.0106991141076928</v>
       </c>
       <c r="BF2" t="n">
-        <v>0.000830765228872155</v>
+        <v>0.00796250761224274</v>
       </c>
       <c r="BG2" t="n">
-        <v>0.0341950264677471</v>
+        <v>-0.00814013673182498</v>
       </c>
       <c r="BH2" t="n">
-        <v>0.0185349492947831</v>
+        <v>0.0180254139557</v>
       </c>
       <c r="BI2" t="n">
-        <v>0.0961004698005625</v>
+        <v>0.061541244804751</v>
       </c>
       <c r="BJ2" t="n">
-        <v>-0.00105540130368376</v>
+        <v>0.10910811424527</v>
       </c>
       <c r="BK2" t="n">
-        <v>0.2047714825147</v>
+        <v>0.172347156687014</v>
       </c>
       <c r="BL2" t="n">
-        <v>-0.00650577522574336</v>
+        <v>0.167025014849186</v>
       </c>
       <c r="BM2" t="n">
-        <v>0.00629826830978408</v>
+        <v>0.0216121444726557</v>
       </c>
       <c r="BN2" t="n">
-        <v>0.0301419262810749</v>
+        <v>-0.00552860648049319</v>
       </c>
       <c r="BO2" t="n">
-        <v>-0.00417905428755339</v>
+        <v>0.020076871297544</v>
       </c>
       <c r="BP2" t="n">
-        <v>-0.0160484565684872</v>
+        <v>-0.000596334236517907</v>
       </c>
       <c r="BQ2" t="n">
-        <v>-0.0000852280322277688</v>
+        <v>-0.024759729936237</v>
       </c>
       <c r="BR2" t="n">
-        <v>-0.0129511453503541</v>
+        <v>0.0536910044030271</v>
       </c>
       <c r="BS2" t="n">
-        <v>-0.00159747613728356</v>
+        <v>-0.00445761944529975</v>
       </c>
       <c r="BT2" t="n">
-        <v>0.0870020442926498</v>
+        <v>0.0950281512954544</v>
       </c>
       <c r="BU2" t="n">
-        <v>-0.00110284023894514</v>
+        <v>-0.00224571915855918</v>
       </c>
       <c r="BV2" t="n">
-        <v>-0.00624691302999958</v>
+        <v>0.0300294346032535</v>
       </c>
       <c r="BW2" t="n">
-        <v>0.103434867884581</v>
+        <v>0.0642001100613866</v>
       </c>
       <c r="BX2" t="n">
-        <v>0.00735383503363507</v>
+        <v>-0.0104722339377632</v>
       </c>
       <c r="BY2" t="n">
-        <v>-0.0225244430405954</v>
+        <v>0.0316717090640184</v>
       </c>
       <c r="BZ2" t="n">
-        <v>-0.023025176281813</v>
+        <v>0.0166802940419907</v>
       </c>
       <c r="CA2" t="n">
-        <v>0.119170049125987</v>
+        <v>-0.0119978458066427</v>
       </c>
       <c r="CB2" t="n">
-        <v>-0.000642888688260679</v>
+        <v>-0.00959634610075521</v>
       </c>
       <c r="CC2" t="n">
-        <v>0.0099512776689592</v>
+        <v>-0.0076156695919673</v>
       </c>
       <c r="CD2" t="n">
-        <v>0.135743600309572</v>
+        <v>0.0211113448920815</v>
       </c>
       <c r="CE2" t="n">
-        <v>-0.0065176101056349</v>
+        <v>0.0287856765743334</v>
       </c>
       <c r="CF2" t="n">
-        <v>-0.00832292079493158</v>
+        <v>-0.00707757535599636</v>
       </c>
       <c r="CG2" t="n">
-        <v>-0.01343006089095</v>
+        <v>0.00255637747753194</v>
       </c>
       <c r="CH2" t="n">
-        <v>0.0129916867258328</v>
+        <v>0.0690205146209864</v>
       </c>
       <c r="CI2" t="n">
-        <v>0.00645824287541141</v>
+        <v>0.0923891379255457</v>
       </c>
       <c r="CJ2" t="n">
-        <v>0.120245866701605</v>
+        <v>0.0697270382035016</v>
       </c>
       <c r="CK2" t="n">
-        <v>0.00702300377402398</v>
+        <v>-0.00706408224606624</v>
       </c>
       <c r="CL2" t="n">
-        <v>0.00987458605750646</v>
+        <v>-0.00811820505428307</v>
       </c>
       <c r="CM2" t="n">
-        <v>0.104735534066873</v>
+        <v>0.0785995494375994</v>
       </c>
       <c r="CN2" t="n">
-        <v>-0.0240595696763997</v>
+        <v>0.0348132299457881</v>
       </c>
       <c r="CO2" t="n">
-        <v>0.0626352621351323</v>
+        <v>0.223715822824603</v>
       </c>
       <c r="CP2" t="n">
-        <v>-0.127641488593322</v>
+        <v>0.0191301841203457</v>
       </c>
       <c r="CQ2" t="n">
-        <v>0.189332007355825</v>
+        <v>0.0466647311035976</v>
       </c>
       <c r="CR2" t="n">
-        <v>0.0562625526786968</v>
+        <v>0.135758835490051</v>
       </c>
       <c r="CS2" t="n">
-        <v>0.0136283392915764</v>
+        <v>-0.0067679343839655</v>
       </c>
       <c r="CT2" t="n">
-        <v>0.249356023124768</v>
+        <v>-0.0120515834738613</v>
       </c>
       <c r="CU2" t="n">
-        <v>-0.000859678431296973</v>
+        <v>-0.0056970412292399</v>
       </c>
       <c r="CV2" t="n">
-        <v>0.145799501504007</v>
+        <v>0.0405137810325646</v>
       </c>
       <c r="CW2" t="n">
-        <v>0.152119145033544</v>
+        <v>0.0212850807670481</v>
       </c>
       <c r="CX2" t="n">
-        <v>0.0705105048130981</v>
+        <v>0.324983612962613</v>
       </c>
       <c r="CY2" t="n">
-        <v>0.0345409079774266</v>
+        <v>0.00447629797530611</v>
       </c>
       <c r="CZ2" t="n">
-        <v>-0.00842065251594071</v>
+        <v>0.00202597855138872</v>
       </c>
       <c r="DA2" t="n">
-        <v>-0.00541838038628684</v>
+        <v>0.0144690657308337</v>
       </c>
       <c r="DB2" t="n">
-        <v>0.035918581267216</v>
+        <v>0.164986849485333</v>
       </c>
       <c r="DC2" t="n">
-        <v>0.0240419657590165</v>
+        <v>-0.00879971387868932</v>
       </c>
       <c r="DD2" t="n">
-        <v>0.0109744867400441</v>
+        <v>0.158970675095345</v>
       </c>
       <c r="DE2" t="n">
-        <v>0.0278916070678241</v>
+        <v>0.00423569705376038</v>
       </c>
       <c r="DF2" t="n">
-        <v>0.0180943367158475</v>
+        <v>0.0250617312528301</v>
       </c>
       <c r="DG2" t="n">
-        <v>0.0605127701684631</v>
+        <v>0.284111699374209</v>
       </c>
       <c r="DH2" t="n">
-        <v>-0.00846478685918872</v>
+        <v>0.0636666369690199</v>
       </c>
       <c r="DI2" t="n">
-        <v>-0.000334856589360832</v>
+        <v>0.00450294499010413</v>
       </c>
       <c r="DJ2" t="n">
-        <v>0.0244104038576813</v>
+        <v>0.257063587483677</v>
       </c>
       <c r="DK2" t="n">
-        <v>-0.00151676522287658</v>
+        <v>0.00266572229242654</v>
       </c>
       <c r="DL2" t="n">
-        <v>0.182462963647733</v>
+        <v>0.0278227383525449</v>
       </c>
       <c r="DM2" t="n">
-        <v>0.0355851304603196</v>
+        <v>0.220933510741433</v>
       </c>
       <c r="DN2" t="n">
-        <v>0.0734981425150578</v>
+        <v>0.0733898876704272</v>
       </c>
       <c r="DO2" t="n">
-        <v>-0.0121521664227525</v>
+        <v>0.0702277463834604</v>
       </c>
       <c r="DP2" t="n">
-        <v>0.116980873172267</v>
+        <v>-0.00866671733296978</v>
       </c>
       <c r="DQ2" t="n">
-        <v>0.0399995905194728</v>
+        <v>-0.00995300954799956</v>
       </c>
       <c r="DR2" t="n">
-        <v>-0.0222366634426961</v>
+        <v>0.125597007734757</v>
       </c>
       <c r="DS2" t="n">
-        <v>0.0243509683230503</v>
+        <v>-0.0087479320501292</v>
       </c>
       <c r="DT2" t="n">
-        <v>-0.00613511906924613</v>
+        <v>-0.00551208274618529</v>
       </c>
       <c r="DU2" t="n">
-        <v>-0.0118242947285556</v>
+        <v>0.110889676585984</v>
       </c>
       <c r="DV2" t="n">
-        <v>-0.00472446717258612</v>
+        <v>-0.00401121776682749</v>
       </c>
       <c r="DW2" t="n">
-        <v>0.0759976411500201</v>
+        <v>0.0142924930465377</v>
       </c>
       <c r="DX2" t="n">
-        <v>0.0235361047719815</v>
+        <v>0.0316696076314511</v>
       </c>
       <c r="DY2" t="n">
-        <v>0.173619946260374</v>
+        <v>0.0515720279475977</v>
       </c>
       <c r="DZ2" t="n">
-        <v>0.115423896054483</v>
-      </c>
-      <c r="EA2" t="n">
-        <v>-0.00418654102039206</v>
-      </c>
+        <v>-0.00173593285644661</v>
+      </c>
+      <c r="EA2"/>
       <c r="EB2" t="n">
-        <v>-0.0387291123777438</v>
+        <v>-0.00450199964770972</v>
       </c>
       <c r="EC2" t="n">
-        <v>0.0453812173641039</v>
+        <v>0.0173415904338212</v>
       </c>
       <c r="ED2" t="n">
-        <v>0.0155453367915745</v>
+        <v>-0.0118898929702016</v>
       </c>
       <c r="EE2" t="n">
-        <v>-0.00171021306032937</v>
+        <v>0.00071687172678009</v>
       </c>
       <c r="EF2" t="n">
-        <v>0.0855779641240968</v>
+        <v>-0.00107610293422413</v>
       </c>
       <c r="EG2" t="n">
-        <v>0.121299291038749</v>
+        <v>0.16185230039953</v>
       </c>
       <c r="EH2" t="n">
-        <v>-0.0251690158847151</v>
+        <v>-0.00628871343232178</v>
       </c>
       <c r="EI2" t="n">
-        <v>0.00874291404039651</v>
+        <v>0.177280915772743</v>
       </c>
       <c r="EJ2" t="n">
-        <v>-0.00154414262321056</v>
+        <v>0.0879472028705173</v>
       </c>
       <c r="EK2" t="n">
-        <v>0.0200996705705383</v>
+        <v>-0.0113992338562445</v>
       </c>
       <c r="EL2" t="n">
-        <v>0.127960242665282</v>
+        <v>0.068114569832133</v>
       </c>
       <c r="EM2" t="n">
-        <v>0.119046311288415</v>
+        <v>-0.739646798600469</v>
       </c>
       <c r="EN2" t="n">
-        <v>0.15088511714125</v>
+        <v>0.0275286249746566</v>
       </c>
       <c r="EO2" t="n">
-        <v>0.0976650944282682</v>
+        <v>0.241365284573072</v>
+      </c>
+      <c r="EP2" t="n">
+        <v>0.00665091347342864</v>
+      </c>
+      <c r="EQ2" t="n">
+        <v>0.138627862294301</v>
+      </c>
+      <c r="ER2" t="n">
+        <v>0.0250239824446958</v>
+      </c>
+      <c r="ES2" t="n">
+        <v>-0.00580578132274533</v>
+      </c>
+      <c r="ET2" t="n">
+        <v>-0.00825396031803091</v>
+      </c>
+      <c r="EU2" t="n">
+        <v>-0.0110091242007338</v>
+      </c>
+      <c r="EV2" t="n">
+        <v>0.0355976433671433</v>
+      </c>
+      <c r="EW2" t="n">
+        <v>0.255256045556998</v>
+      </c>
+      <c r="EX2" t="n">
+        <v>0.209212087599447</v>
+      </c>
+      <c r="EY2" t="n">
+        <v>0.156497627545887</v>
+      </c>
+      <c r="EZ2" t="n">
+        <v>0.017563504092658</v>
+      </c>
+      <c r="FA2" t="n">
+        <v>0.115780004402048</v>
+      </c>
+      <c r="FB2" t="n">
+        <v>0.00870594180360536</v>
+      </c>
+      <c r="FC2" t="n">
+        <v>0.076791433319674</v>
+      </c>
+      <c r="FD2" t="n">
+        <v>-0.00516417402200463</v>
+      </c>
+      <c r="FE2" t="n">
+        <v>0.0407738404692603</v>
+      </c>
+      <c r="FF2" t="n">
+        <v>0.00499523323764764</v>
+      </c>
+      <c r="FG2"/>
+      <c r="FH2" t="n">
+        <v>0.117760020677719</v>
+      </c>
+      <c r="FI2" t="n">
+        <v>0.147588904238383</v>
+      </c>
+      <c r="FJ2" t="n">
+        <v>0.0333330374075334</v>
+      </c>
+      <c r="FK2" t="n">
+        <v>-0.00441895836298513</v>
+      </c>
+      <c r="FL2" t="n">
+        <v>-0.0126771610347124</v>
+      </c>
+      <c r="FM2" t="n">
+        <v>0.0591896079496654</v>
+      </c>
+      <c r="FN2" t="n">
+        <v>0.000339769003218122</v>
+      </c>
+      <c r="FO2" t="n">
+        <v>0.04061398679882</v>
+      </c>
+      <c r="FP2" t="n">
+        <v>0.0307623723041562</v>
+      </c>
+      <c r="FQ2" t="n">
+        <v>0.0276464394642444</v>
+      </c>
+      <c r="FR2" t="n">
+        <v>0.218736277122264</v>
+      </c>
+      <c r="FS2" t="n">
+        <v>0.0169594258029628</v>
+      </c>
+      <c r="FT2" t="n">
+        <v>0.11171958372138</v>
+      </c>
+      <c r="FU2" t="n">
+        <v>0.0680150585482112</v>
       </c>
     </row>
   </sheetData>

</xml_diff>